<commit_message>
Un seul axe : modèles d'import à jour, données de référence ComptaBB retirées, CLAUDE.md de ComptaJLC
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V8s2z31P3cgDQRDppUofdK
</commit_message>
<xml_diff>
--- a/Imports/modeles/Budget.xlsx
+++ b/Imports/modeles/Budget.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Budget" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -431,7 +431,6 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -452,15 +451,10 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Axe 1</t>
+          <t>Anal</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Axe 2</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Montant</t>
         </is>

</xml_diff>